<commit_message>
Improve Q4 bounds and certify Q5 plan
</commit_message>
<xml_diff>
--- a/deliverables/result3.xlsx
+++ b/deliverables/result3.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R38a3424497a344cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R75e7bf0b2c6f43b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44,21 +44,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">干扰的导弹编号</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">FY1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">FY2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">FY3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">FY4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">FY5</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">注：以x轴为正向，逆时针方向为正，取值0~360（度）。</x:t>
@@ -368,8 +353,8 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="3" t="s">
-        <x:v>12</x:v>
+      <x:c r="A2" s="3" t="str">
+        <x:v>FY1</x:v>
       </x:c>
       <x:c r="B2" s="4" t="n">
         <x:v>179.84702991159443</x:v>
@@ -377,7 +362,7 @@
       <x:c r="C2" s="4" t="n">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="D2" s="6">
+      <x:c r="D2" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E2" s="4" t="n">
@@ -406,8 +391,8 @@
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="3" t="s">
-        <x:v>12</x:v>
+      <x:c r="A3" s="3" t="str">
+        <x:v>FY1</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
         <x:v>179.84702991159443</x:v>
@@ -415,7 +400,7 @@
       <x:c r="C3" s="4" t="n">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="D3" s="6">
+      <x:c r="D3" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E3" s="4" t="n">
@@ -444,8 +429,8 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="3" t="s">
-        <x:v>12</x:v>
+      <x:c r="A4" s="3" t="str">
+        <x:v>FY1</x:v>
       </x:c>
       <x:c r="B4" s="4" t="n">
         <x:v>179.84702991159443</x:v>
@@ -453,7 +438,7 @@
       <x:c r="C4" s="4" t="n">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="D4" s="6">
+      <x:c r="D4" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E4" s="4" t="n">
@@ -482,8 +467,8 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="3" t="s">
-        <x:v>13</x:v>
+      <x:c r="A5" s="3" t="str">
+        <x:v>FY2</x:v>
       </x:c>
       <x:c r="B5" s="4" t="n">
         <x:v>308.64053756976966</x:v>
@@ -491,7 +476,7 @@
       <x:c r="C5" s="4" t="n">
         <x:v>134.27872322197402</x:v>
       </x:c>
-      <x:c r="D5" s="6">
+      <x:c r="D5" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E5" s="4" t="n">
@@ -520,30 +505,50 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="3" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B6" s="4"/>
-      <x:c r="C6" s="4"/>
-      <x:c r="D6" s="6">
+      <x:c r="A6" s="3" t="str">
+        <x:v>FY2</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="n">
+        <x:v>308.64053756976966</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="n">
+        <x:v>134.27872322197402</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E6" s="4"/>
-      <x:c r="F6" s="4"/>
-      <x:c r="G6" s="4"/>
-      <x:c r="H6" s="4"/>
-      <x:c r="I6" s="4"/>
-      <x:c r="J6" s="4"/>
-      <x:c r="K6" s="4"/>
-      <x:c r="L6"/>
+      <x:c r="E6" s="4" t="n">
+        <x:v>12831.069750456982</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="n">
+        <x:v>360.4462421380522</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="n">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="n">
+        <x:v>13114.633517172728</x:v>
+      </x:c>
+      <x:c r="I6" s="4" t="n">
+        <x:v>5.747037744256204</x:v>
+      </x:c>
+      <x:c r="J6" s="4" t="n">
+        <x:v>1343.958168474142</x:v>
+      </x:c>
+      <x:c r="K6" s="4" t="n">
+        <x:v>2.094496970681025</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>M1</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="3" t="s">
-        <x:v>13</x:v>
+      <x:c r="A7" s="3" t="str">
+        <x:v>FY2</x:v>
       </x:c>
       <x:c r="B7" s="4"/>
       <x:c r="C7" s="4"/>
-      <x:c r="D7" s="6">
+      <x:c r="D7" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E7" s="4"/>
@@ -556,8 +561,8 @@
       <x:c r="L7"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="3" t="s">
-        <x:v>14</x:v>
+      <x:c r="A8" s="3" t="str">
+        <x:v>FY3</x:v>
       </x:c>
       <x:c r="B8" s="4" t="n">
         <x:v>74.8074657707454</x:v>
@@ -565,7 +570,7 @@
       <x:c r="C8" s="4" t="n">
         <x:v>139.56614835243784</x:v>
       </x:c>
-      <x:c r="D8" s="6">
+      <x:c r="D8" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E8" s="4" t="n">
@@ -594,8 +599,8 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="3" t="s">
-        <x:v>14</x:v>
+      <x:c r="A9" s="3" t="str">
+        <x:v>FY3</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:v>74.8074657707454</x:v>
@@ -603,7 +608,7 @@
       <x:c r="C9" s="4" t="n">
         <x:v>139.56614835243784</x:v>
       </x:c>
-      <x:c r="D9" s="6">
+      <x:c r="D9" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E9" s="4" t="n">
@@ -632,12 +637,12 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="3" t="s">
-        <x:v>14</x:v>
+      <x:c r="A10" s="3" t="str">
+        <x:v>FY3</x:v>
       </x:c>
       <x:c r="B10" s="4"/>
       <x:c r="C10" s="4"/>
-      <x:c r="D10" s="6">
+      <x:c r="D10" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E10" s="4"/>
@@ -650,8 +655,8 @@
       <x:c r="L10"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="3" t="s">
-        <x:v>15</x:v>
+      <x:c r="A11" s="3" t="str">
+        <x:v>FY4</x:v>
       </x:c>
       <x:c r="B11" s="4" t="n">
         <x:v>267.6871810269418</x:v>
@@ -659,7 +664,7 @@
       <x:c r="C11" s="4" t="n">
         <x:v>111.7021843781944</x:v>
       </x:c>
-      <x:c r="D11" s="6">
+      <x:c r="D11" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E11" s="4" t="n">
@@ -688,8 +693,8 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="3" t="s">
-        <x:v>15</x:v>
+      <x:c r="A12" s="3" t="str">
+        <x:v>FY4</x:v>
       </x:c>
       <x:c r="B12" s="4" t="n">
         <x:v>267.6871810269418</x:v>
@@ -697,55 +702,75 @@
       <x:c r="C12" s="4" t="n">
         <x:v>111.7021843781944</x:v>
       </x:c>
-      <x:c r="D12" s="6">
+      <x:c r="D12" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E12" s="4" t="n">
-        <x:v>10956.494182304323</x:v>
+        <x:v>10975.089713658917</x:v>
       </x:c>
       <x:c r="F12" s="4" t="n">
-        <x:v>922.8099044035494</x:v>
+        <x:v>1383.2292979117642</x:v>
       </x:c>
       <x:c r="G12" s="4" t="n">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="H12" s="4" t="n">
+        <x:v>10921.208004987442</x:v>
+      </x:c>
+      <x:c r="I12" s="4" t="n">
+        <x:v>49.135468881328734</x:v>
+      </x:c>
+      <x:c r="J12" s="4" t="n">
+        <x:v>1099.9108497625098</x:v>
+      </x:c>
+      <x:c r="K12" s="4" t="n">
+        <x:v>3.3403124946328404</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>M1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="3" t="str">
+        <x:v>FY4</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="n">
+        <x:v>267.6871810269418</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="n">
+        <x:v>111.7021843781944</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="n">
+        <x:v>10956.494182304323</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="n">
+        <x:v>922.8099044035494</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="n">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="n">
         <x:v>10904.943198910172</x:v>
       </x:c>
-      <x:c r="I12" s="4" t="n">
+      <x:c r="I13" s="4" t="n">
         <x:v>-353.57591412925376</x:v>
       </x:c>
-      <x:c r="J12" s="4" t="n">
+      <x:c r="J13" s="4" t="n">
         <x:v>1159.1674881267104</x:v>
       </x:c>
-      <x:c r="K12" s="4" t="n">
+      <x:c r="K13" s="4" t="n">
         <x:v>2.712016729925633</x:v>
       </x:c>
-      <x:c r="L12" t="str">
+      <x:c r="L13" t="str">
         <x:v>M3</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="3" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B13" s="4"/>
-      <x:c r="C13" s="4"/>
-      <x:c r="D13" s="6">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E13" s="4"/>
-      <x:c r="F13" s="4"/>
-      <x:c r="G13" s="4"/>
-      <x:c r="H13" s="4"/>
-      <x:c r="I13" s="4"/>
-      <x:c r="J13" s="4"/>
-      <x:c r="K13" s="4"/>
-      <x:c r="L13"/>
-    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="A14" s="3" t="str">
+        <x:v>FY5</x:v>
       </x:c>
       <x:c r="B14" s="4" t="n">
         <x:v>118.23767394874588</x:v>
@@ -753,7 +778,7 @@
       <x:c r="C14" s="4" t="n">
         <x:v>139.99999434843764</x:v>
       </x:c>
-      <x:c r="D14" s="6">
+      <x:c r="D14" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E14" s="4" t="n">
@@ -782,8 +807,8 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="A15" s="3" t="str">
+        <x:v>FY5</x:v>
       </x:c>
       <x:c r="B15" s="4" t="n">
         <x:v>118.23767394874588</x:v>
@@ -791,7 +816,7 @@
       <x:c r="C15" s="4" t="n">
         <x:v>139.99999434843764</x:v>
       </x:c>
-      <x:c r="D15" s="6">
+      <x:c r="D15" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E15" s="4" t="n">
@@ -820,8 +845,8 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="3" t="s">
-        <x:v>16</x:v>
+      <x:c r="A16" s="3" t="str">
+        <x:v>FY5</x:v>
       </x:c>
       <x:c r="B16" s="4" t="n">
         <x:v>118.23767394874588</x:v>
@@ -829,7 +854,7 @@
       <x:c r="C16" s="4" t="n">
         <x:v>139.99999434843764</x:v>
       </x:c>
-      <x:c r="D16" s="6">
+      <x:c r="D16" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E16" s="4" t="n">
@@ -860,7 +885,7 @@
     <x:row r="18" ht="60" customHeight="1">
       <x:c r="A18" s="1"/>
       <x:c r="B18" s="2" t="s">
-        <x:v>17</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>